<commit_message>
fix: job status/cancel role checks, PayNow payee name, banner artwork, progress log
</commit_message>
<xml_diff>
--- a/marketing/TCG-Express-launch-incentive-budget.xlsx
+++ b/marketing/TCG-Express-launch-incentive-budget.xlsx
@@ -599,11 +599,11 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>DB 실측 2026-08-29: approved 57 + pending 14 (rejected 3 제외)</t>
+          <t>DB 실측 8/29: approved 57(중 테스트 5) + pending 14. 실사용 66명</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>DB 실측 — driver_status='approved'. 전원 배송 실적 0건</t>
+          <t>approved 57 - 테스트계정 5. 이 중 54명이 배송 0건, 2명 1~4건, 1명 5건+(웰컴보너스 정상 지급됨)</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -672,7 +672,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>★ 하향 조정. 승인 드라이버 57명이 이미 대기 중인데 지금까지 완료 배송은 6건뿐 — 병목은 드라이버가 아니라 수요</t>
+          <t>실측 근거: 실고객 주문은 82건 중 9건뿐, 최근 주문 8/9. 병목은 드라이버가 아니라 수요</t>
         </is>
       </c>
       <c r="D9" s="5" t="n"/>

</xml_diff>